<commit_message>
Rev 8: third stomp (SW3) + STOMP3 to GP22, boards/BOM/fab package updated
CONTROL: SW3 at (69,96); SW1/SW2 outboard to 23.28/114.72 (1.800in pitch);
LED4/LED5 follow; C7 +1.5mm east; 3 GND stitch vias cleared from new pad rows;
/POT3_W detoured around SW2's new COM pad; stomp silk now A/B/C; STOMP3 on
spare J1 pin 15. Fixes schematic pin1/pin3 inversion on SW1/SW2 (GND belongs
on N.O.; PCB was already right). DRC 0 errors.

MAIN: R175 10k pullup + C125 100n added; STOMP3 routed J10.15 -> GP22 (Pico
pad 29). DRC/ERC at pre-existing baselines. BOM.xlsx updated (SW qty 3, R/C
qty bumps, stale Suntsu README lines replaced). Fab package regenerated both
boards: Glitchwave567_PCBWay_Release_20260921.zip, README_PCBWAY rev 0.6.

Enclosure drill template still stale: needs three D12.2 at centreline +/-45.72mm.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01ArRoxLtCyE7DZoHE3DcYLs
</commit_message>
<xml_diff>
--- a/hardware/BOM.xlsx
+++ b/hardware/BOM.xlsx
@@ -929,11 +929,11 @@
         <v>10</v>
       </c>
       <c r="B11" s="3" t="n">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>C101,C106,C107,C111,C121,C122,C123,C124,C20,C21,C22,C23,C30,C31,C33,C34,C35,C40,C49,C50,C63,C64,C65,C66,C67,C70,C71,C73,C76,C77,C78,C83,C84,C85,C91,C910,C911,C93,C94,C95,C96,C97,C98,C99</t>
+          <t>C101,C106,C107,C111,C121,C122,C123,C124,C125,C20,C21,C22,C23,C30,C31,C33,C34,C35,C40,C49,C50,C63,C64,C65,C66,C67,C70,C71,C73,C76,C77,C78,C83,C84,C85,C91,C910,C911,C93,C94,C95,C96,C97,C98,C99</t>
         </is>
       </c>
       <c r="D11" s="3" t="inlineStr">
@@ -3181,11 +3181,11 @@
         <v>61</v>
       </c>
       <c r="B62" s="3" t="n">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C62" s="3" t="inlineStr">
         <is>
-          <t>R106A,R107A,R110,R111,R112A,R113A,R117A,R121A,R125A,R142,R145,R146,R147,R148,R161,R162,R163,R164,R165,R166,R167,R168,R169,R171,R172,R174,R25,R33,R35,R48,R49,R51,R64,R68,R76,R79,R83,R88,R90,R92</t>
+          <t>R106A,R107A,R110,R111,R112A,R113A,R117A,R121A,R125A,R142,R145,R146,R147,R148,R161,R162,R163,R164,R165,R166,R167,R168,R169,R171,R172,R174,R175,R25,R33,R35,R48,R49,R51,R64,R68,R76,R79,R83,R88,R90,R92</t>
         </is>
       </c>
       <c r="D62" s="3" t="inlineStr">
@@ -5239,16 +5239,16 @@
         <v>10</v>
       </c>
       <c r="B11" s="3" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>SW1,SW2</t>
+          <t>SW1,SW2,SW3</t>
         </is>
       </c>
       <c r="D11" s="3" t="inlineStr">
         <is>
-          <t>Alpha SF12011F-0102-20R-M-011 (momentary, TAP/BYP + TAP/TEMPO)</t>
+          <t>Alpha SF12011F-0102-20R-M-011 (momentary, stomps A/B/C)</t>
         </is>
       </c>
       <c r="E11" s="3" t="inlineStr">
@@ -5273,7 +5273,7 @@
       </c>
       <c r="I11" s="3" t="inlineStr">
         <is>
-          <t>2026-09-05: switched from Suntsu SSWFS-S01 (unsourceable) to Alpha SF12011F-0102-20R-M-011. Both SW1 and SW2 kept MOMENTARY (not latching) to preserve the STARVE gesture (both-held) and existing 2-switch/5-gesture firmware in stomps.c - a latching bypass switch was considered and rejected. "011F" prefix = Alpha's genuine PCB-mount (PC-pin) terminal type per their SF12 series datasheet, confirmed board-mountable with no panel cutouts (matches project's existing no-cutout architecture) - the E-Switch FS5700 alternate looked into earlier was rejected because it uses rear solder lugs, not PCB pins, and cannot be machine-assembled. VERIFIED from Alpha's own SF12 series datasheet (user-supplied PDF, page 3, SF12011F-0102-20R-M-011 outline drawing): terminals in a straight row, 2.5mm pitch, ~1.0mm pin width; pinout Pin 1=N.O., Pin 2=COM, Pin 3=N.C. (wiring diagram: PUSH 1-2 ON, FREE 2-3 ON). Pin 1 (N.O.) wired to GND, pin 2 (COM) wired to the existing GPIO/pullup net, pin 3 (N.C.) left genuinely unconnected. Thread M12x0.75 vs prior M12x1.0 spec - panel hole stays D12.2 (M12 nominal OD unaffected by thread pitch), no enclosure change needed. Body 13.4mm dia, ~12mm deep below panel - fits existing 15.0+/-1.0mm enclosure depth budget. Since the real part's pin pitch/positions differ from the old SSWFS-S01 footprint, the PCB routing at SW1/SW2 was re-run (new footprint, corrected pinout, existing traces rerouted to reach the new pad positions) - DRC and ERC both clean (0 errors) as of 2026-09-05. No longer DNP - PCBWay turnkey should be able to source and place this by MPN.</t>
+          <t>2026-09-05: switched from Suntsu SSWFS-S01 (unsourceable) to Alpha SF12011F-0102-20R-M-011. Both SW1 and SW2 kept MOMENTARY (not latching) to preserve the STARVE gesture (both-held) and existing 2-switch/5-gesture firmware in stomps.c - a latching bypass switch was considered and rejected. "011F" prefix = Alpha's genuine PCB-mount (PC-pin) terminal type per their SF12 series datasheet, confirmed board-mountable with no panel cutouts (matches project's existing no-cutout architecture) - the E-Switch FS5700 alternate looked into earlier was rejected because it uses rear solder lugs, not PCB pins, and cannot be machine-assembled. VERIFIED from Alpha's own SF12 series datasheet (user-supplied PDF, page 3, SF12011F-0102-20R-M-011 outline drawing): terminals in a straight row, 2.5mm pitch, ~1.0mm pin width; pinout Pin 1=N.O., Pin 2=COM, Pin 3=N.C. (wiring diagram: PUSH 1-2 ON, FREE 2-3 ON). Pin 1 (N.O.) wired to GND, pin 2 (COM) wired to the existing GPIO/pullup net, pin 3 (N.C.) left genuinely unconnected. Thread M12x0.75 vs prior M12x1.0 spec - panel hole stays D12.2 (M12 nominal OD unaffected by thread pitch), no enclosure change needed. Body 13.4mm dia, ~12mm deep below panel - fits existing 15.0+/-1.0mm enclosure depth budget. Since the real part's pin pitch/positions differ from the old SSWFS-S01 footprint, the PCB routing at SW1/SW2 was re-run (new footprint, corrected pinout, existing traces rerouted to reach the new pad positions) - DRC and ERC both clean (0 errors) as of 2026-09-05. No longer DNP - PCBWay turnkey should be able to source and place this by MPN. | Rev8 2026-09-21: third stomp SW3 added at board centre x=69.00, SW1/SW2 moved outboard to 23.28/114.72 (1.800in pitch), same part/wiring (pin1 N.O.-&gt;GND, pin2 COM-&gt;STOMP3 via J1 pin 15 -&gt; GP22).</t>
         </is>
       </c>
       <c r="J11" s="3" t="n"/>
@@ -5407,21 +5407,21 @@
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>Stomps: Suntsu SSWFS-S01-AC09-HWH via Digi-Key (PCBWay buys from DK/Mouser for turnkey).</t>
+          <t>Stomps: 3x Alpha SF12011F-0102-20R-M-011 (SW1,SW2,SW3) - Alpha Taiwan direct, PCBWay turnkey sources by MPN (not LCSC/DK stocked). Rev8 2026-09-21 added SW3.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">  CONFIRM at order time that PCBWay will purchase Digi-Key MARKETPLACE items; if not, use SSWFS-S01-AC05-HWH (DK own stock,</t>
+          <t xml:space="preserve">  (Suntsu SSWFS-S01 references are obsolete - superseded 2026-09-05 by the Alpha part above.)</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">  solder lug) shipped loose + 2 wires per stomp to the same control-board pads.</t>
+          <t xml:space="preserve">  Stomp wiring: pin 1 (N.O.) to GND, pin 2 (COM) to STOMP net, pin 3 (N.C.) unconnected.</t>
         </is>
       </c>
     </row>

</xml_diff>